<commit_message>
The reference note on the shelter called it a bus stop
Regenerates the tables the note is baked into, and the workbook that
draws from them. Numbers are unchanged - Table 5.5 and Table 5.7 check
out to the decimal against the dissertation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tables/summary_all_objects_accuracy_f1_EN.xlsx
+++ b/docs/tables/summary_all_objects_accuracy_f1_EN.xlsx
@@ -804,7 +804,7 @@
       </c>
       <c r="AI2" s="5" t="inlineStr">
         <is>
-          <t>incomplete reference: the bus stop's far side (away from the road) wasn't scanned; part of the reference is a merge of 2 scans that don't align perfectly in places</t>
+          <t>incomplete reference: the bus shelter's far side (away from the road) wasn't scanned; part of the reference is a merge of 2 scans that don't align perfectly in places</t>
         </is>
       </c>
     </row>
@@ -2926,8 +2926,8 @@
   </sheetData>
   <mergeCells count="48">
     <mergeCell ref="AI10:AI13"/>
+    <mergeCell ref="E18:E21"/>
     <mergeCell ref="C14:C17"/>
-    <mergeCell ref="E18:E21"/>
     <mergeCell ref="E14:E17"/>
     <mergeCell ref="AH18:AH21"/>
     <mergeCell ref="B22:B25"/>
@@ -3004,6 +3004,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>

</xml_diff>